<commit_message>
Mis à jour demo
Nettoyage des prints
</commit_message>
<xml_diff>
--- a/demo/MTG.xlsx
+++ b/demo/MTG.xlsx
@@ -949,7 +949,7 @@
         </is>
       </c>
       <c r="AZ2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="BA2" t="inlineStr">
         <is>
@@ -1223,7 +1223,7 @@
         </is>
       </c>
       <c r="AZ3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="BA3" t="inlineStr">
         <is>
@@ -1318,7 +1318,7 @@
         <v>0.5278586297772488</v>
       </c>
       <c r="W4" t="n">
-        <v>5.451217609071717</v>
+        <v>5.258295729711735</v>
       </c>
       <c r="X4" t="n">
         <v>0</v>
@@ -1327,13 +1327,13 @@
         <v>0</v>
       </c>
       <c r="Z4" t="n">
-        <v>18.60942576789385</v>
+        <v>17.95082696476085</v>
       </c>
       <c r="AA4" t="n">
-        <v>0.707812064001736</v>
+        <v>0.6827621681044143</v>
       </c>
       <c r="AB4" t="n">
-        <v>0.6827621681044147</v>
+        <v>0.6585988031330005</v>
       </c>
       <c r="AC4" t="inlineStr">
         <is>
@@ -1350,7 +1350,7 @@
         <v>1</v>
       </c>
       <c r="AG4" t="n">
-        <v>0.707812064001736</v>
+        <v>0.6827621681044143</v>
       </c>
       <c r="AH4" t="n">
         <v>1.5</v>
@@ -1382,10 +1382,10 @@
         <v>0</v>
       </c>
       <c r="AQ4" t="n">
-        <v>66.66666666666667</v>
+        <v>64.30729311999421</v>
       </c>
       <c r="AR4" t="n">
-        <v>20</v>
+        <v>19.29218793599826</v>
       </c>
       <c r="AS4" t="n">
         <v>0.07078120640017346</v>
@@ -1413,7 +1413,7 @@
         <v>0.002218195854645766</v>
       </c>
       <c r="AZ4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="BA4" t="n">
         <v>1.45574</v>
@@ -1685,7 +1685,7 @@
         </is>
       </c>
       <c r="AZ5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="BA5" t="inlineStr">
         <is>
@@ -1780,7 +1780,7 @@
         <v>1.049772235680382</v>
       </c>
       <c r="W6" t="n">
-        <v>5.647618296916117</v>
+        <v>5.454458688673748</v>
       </c>
       <c r="X6" t="n">
         <v>0</v>
@@ -1789,13 +1789,13 @@
         <v>0</v>
       </c>
       <c r="Z6" t="n">
-        <v>18.65531712817264</v>
+        <v>18.01726874057487</v>
       </c>
       <c r="AA6" t="n">
-        <v>0.6840391757631465</v>
+        <v>0.6606436960642128</v>
       </c>
       <c r="AB6" t="n">
-        <v>0.6606436960642111</v>
+        <v>0.6380483875977669</v>
       </c>
       <c r="AC6" t="inlineStr">
         <is>
@@ -1812,7 +1812,7 @@
         <v>1</v>
       </c>
       <c r="AG6" t="n">
-        <v>0.6840391757631465</v>
+        <v>0.6606436960642128</v>
       </c>
       <c r="AH6" t="n">
         <v>1.5</v>
@@ -1844,10 +1844,10 @@
         <v>0</v>
       </c>
       <c r="AQ6" t="n">
-        <v>66.66666666666667</v>
+        <v>64.38653608078951</v>
       </c>
       <c r="AR6" t="n">
-        <v>20</v>
+        <v>19.31596082423685</v>
       </c>
       <c r="AS6" t="n">
         <v>0.06840391757631474</v>
@@ -1875,7 +1875,7 @@
         <v>0.008773134791588384</v>
       </c>
       <c r="AZ6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="BA6" t="n">
         <v>2.240171</v>
@@ -2147,7 +2147,7 @@
         </is>
       </c>
       <c r="AZ7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="BA7" t="inlineStr">
         <is>
@@ -2242,7 +2242,7 @@
         <v>1.842407650978477</v>
       </c>
       <c r="W8" t="n">
-        <v>5.178476312455444</v>
+        <v>4.985913362964966</v>
       </c>
       <c r="X8" t="n">
         <v>0</v>
@@ -2251,13 +2251,13 @@
         <v>0</v>
       </c>
       <c r="Z8" t="n">
-        <v>18.54024475823615</v>
+        <v>17.85082107460661</v>
       </c>
       <c r="AA8" t="n">
-        <v>0.7437050509522223</v>
+        <v>0.7160501908116323</v>
       </c>
       <c r="AB8" t="n">
-        <v>0.7160501908116307</v>
+        <v>0.689423683629535</v>
       </c>
       <c r="AC8" t="inlineStr">
         <is>
@@ -2274,7 +2274,7 @@
         <v>1</v>
       </c>
       <c r="AG8" t="n">
-        <v>0.7437050509522223</v>
+        <v>0.7160501908116323</v>
       </c>
       <c r="AH8" t="n">
         <v>1.5</v>
@@ -2306,10 +2306,10 @@
         <v>0</v>
       </c>
       <c r="AQ8" t="n">
-        <v>66.66666666666667</v>
+        <v>64.18764983015926</v>
       </c>
       <c r="AR8" t="n">
-        <v>20</v>
+        <v>19.25629494904778</v>
       </c>
       <c r="AS8" t="n">
         <v>0.07437050509522231</v>
@@ -2337,7 +2337,7 @@
         <v>0.02702315760287949</v>
       </c>
       <c r="AZ8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="BA8" t="n">
         <v>3.124146</v>
@@ -2609,7 +2609,7 @@
         </is>
       </c>
       <c r="AZ9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="BA9" t="inlineStr">
         <is>
@@ -2704,7 +2704,7 @@
         <v>2.853576792270807</v>
       </c>
       <c r="W10" t="n">
-        <v>4.667771046361761</v>
+        <v>4.475988359710937</v>
       </c>
       <c r="X10" t="n">
         <v>0</v>
@@ -2713,13 +2713,13 @@
         <v>0</v>
       </c>
       <c r="Z10" t="n">
-        <v>18.39029944950411</v>
+        <v>17.63470518369536</v>
       </c>
       <c r="AA10" t="n">
-        <v>0.8217313349175797</v>
+        <v>0.7879692155783111</v>
       </c>
       <c r="AB10" t="n">
-        <v>0.7879692155783096</v>
+        <v>0.7555942658087533</v>
       </c>
       <c r="AC10" t="inlineStr">
         <is>
@@ -2736,7 +2736,7 @@
         <v>1</v>
       </c>
       <c r="AG10" t="n">
-        <v>0.8217313349175797</v>
+        <v>0.7879692155783111</v>
       </c>
       <c r="AH10" t="n">
         <v>1.5</v>
@@ -2768,10 +2768,10 @@
         <v>0</v>
       </c>
       <c r="AQ10" t="n">
-        <v>66.66666666666667</v>
+        <v>63.9275622169414</v>
       </c>
       <c r="AR10" t="n">
-        <v>20</v>
+        <v>19.17826866508242</v>
       </c>
       <c r="AS10" t="n">
         <v>0.08217313349175812</v>
@@ -2799,7 +2799,7 @@
         <v>0.06482518513852682</v>
       </c>
       <c r="AZ10" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="BA10" t="n">
         <v>5.58545</v>
@@ -3071,7 +3071,7 @@
         </is>
       </c>
       <c r="AZ11" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="BA11" t="inlineStr">
         <is>
@@ -3166,7 +3166,7 @@
         <v>3.900377027728756</v>
       </c>
       <c r="W12" t="n">
-        <v>3.07445026731027</v>
+        <v>2.886666058278094</v>
       </c>
       <c r="X12" t="n">
         <v>0</v>
@@ -3175,13 +3175,13 @@
         <v>0</v>
       </c>
       <c r="Z12" t="n">
-        <v>17.63145458091985</v>
+        <v>16.55454376282379</v>
       </c>
       <c r="AA12" t="n">
-        <v>1.22157909678247</v>
+        <v>1.146966322297676</v>
       </c>
       <c r="AB12" t="n">
-        <v>1.146966322297677</v>
+        <v>1.076910818096062</v>
       </c>
       <c r="AC12" t="inlineStr">
         <is>
@@ -3198,7 +3198,7 @@
         <v>1</v>
       </c>
       <c r="AG12" t="n">
-        <v>1.22157909678247</v>
+        <v>1.146966322297676</v>
       </c>
       <c r="AH12" t="n">
         <v>1.5</v>
@@ -3230,10 +3230,10 @@
         <v>0</v>
       </c>
       <c r="AQ12" t="n">
-        <v>66.66666666666667</v>
+        <v>62.59473634405843</v>
       </c>
       <c r="AR12" t="n">
-        <v>20</v>
+        <v>18.77842090321753</v>
       </c>
       <c r="AS12" t="n">
         <v>0.1221579096782471</v>
@@ -3261,7 +3261,7 @@
         <v>0.1211093900748481</v>
       </c>
       <c r="AZ12" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="BA12" t="n">
         <v>10.683281</v>
@@ -3533,7 +3533,7 @@
         </is>
       </c>
       <c r="AZ13" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="BA13" t="inlineStr">
         <is>
@@ -3628,7 +3628,7 @@
         <v>4.704752754993121</v>
       </c>
       <c r="W14" t="n">
-        <v>1.291618033556523</v>
+        <v>1.118434550318946</v>
       </c>
       <c r="X14" t="n">
         <v>0</v>
@@ -3637,13 +3637,13 @@
         <v>0</v>
       </c>
       <c r="Z14" t="n">
-        <v>14.99625943315017</v>
+        <v>12.98552222083664</v>
       </c>
       <c r="AA14" t="n">
-        <v>2.681651676242236</v>
+        <v>2.322088890607597</v>
       </c>
       <c r="AB14" t="n">
-        <v>2.322088890607597</v>
+        <v>2.01073721231353</v>
       </c>
       <c r="AC14" t="inlineStr">
         <is>
@@ -3660,7 +3660,7 @@
         <v>1</v>
       </c>
       <c r="AG14" t="n">
-        <v>2.681651676242236</v>
+        <v>2.322088890607597</v>
       </c>
       <c r="AH14" t="n">
         <v>1.5</v>
@@ -3692,10 +3692,10 @@
         <v>0</v>
       </c>
       <c r="AQ14" t="n">
-        <v>66.66666666666667</v>
+        <v>57.72782774585922</v>
       </c>
       <c r="AR14" t="n">
-        <v>20</v>
+        <v>17.31834832375776</v>
       </c>
       <c r="AS14" t="n">
         <v>0.2681651676242238</v>
@@ -3723,7 +3723,7 @@
         <v>0.1762131227885508</v>
       </c>
       <c r="AZ14" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="BA14" t="n">
         <v>18.274131</v>
@@ -3995,7 +3995,7 @@
         </is>
       </c>
       <c r="AZ15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="BA15" t="inlineStr">
         <is>
@@ -4185,7 +4185,7 @@
         <v>0.1996756274979211</v>
       </c>
       <c r="AZ16" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="BA16" t="n">
         <v>25.705583</v>
@@ -4457,7 +4457,7 @@
         </is>
       </c>
       <c r="AZ17" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="BA17" t="inlineStr">
         <is>
@@ -4647,7 +4647,7 @@
         <v>0.1762131227885509</v>
       </c>
       <c r="AZ18" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="BA18" t="n">
         <v>28.86908</v>
@@ -4919,7 +4919,7 @@
         </is>
       </c>
       <c r="AZ19" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="BA19" t="inlineStr">
         <is>
@@ -5109,7 +5109,7 @@
         <v>0.1211093900748481</v>
       </c>
       <c r="AZ20" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="BA20" t="n">
         <v>25.7056</v>
@@ -5381,7 +5381,7 @@
         </is>
       </c>
       <c r="AZ21" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="BA21" t="inlineStr">
         <is>
@@ -5571,7 +5571,7 @@
         <v>0.06482518513852684</v>
       </c>
       <c r="AZ22" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="BA22" t="n">
         <v>18.273897</v>
@@ -5843,7 +5843,7 @@
         </is>
       </c>
       <c r="AZ23" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="BA23" t="inlineStr">
         <is>
@@ -6033,7 +6033,7 @@
         <v>0.02702315760287954</v>
       </c>
       <c r="AZ24" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="BA24" t="n">
         <v>10.68338</v>
@@ -6305,7 +6305,7 @@
         </is>
       </c>
       <c r="AZ25" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="BA25" t="inlineStr">
         <is>
@@ -6495,7 +6495,7 @@
         <v>0.00877313479158839</v>
       </c>
       <c r="AZ26" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="BA26" t="n">
         <v>5.585384</v>
@@ -6767,7 +6767,7 @@
         </is>
       </c>
       <c r="AZ27" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="BA27" t="inlineStr">
         <is>
@@ -6957,7 +6957,7 @@
         <v>0.002218195854645766</v>
       </c>
       <c r="AZ28" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="BA28" t="n">
         <v>3.124212</v>

</xml_diff>